<commit_message>
feat(magazine): dynamic related-articles + query-index Members Only
- Related articles (article pages) now use the dynamic article-list block
  instead of static cards-related; article-list excludes the current page so
  an article never lists itself.
- Members Only (magazine landing) is now query-index driven: article-list
  gains a 'members' mode that filters the magazine index by a members flag and
  renders locked secure cards (lock badge, grey text, READ MORE, image below).
- Fix oversized Members Only cards: fixed ~388px width + 200px image height
  (was stretching full-width with 13/10 ratio).
- helix-query.yaml: add members field to magazine index; drop members-only
  exclude so member pages are indexed (they live 2 levels deep, so the All
  Articles listing still excludes them).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-magazine-article.report.xlsx
+++ b/tools/importer/reports/import-magazine-article.report.xlsx
@@ -49,7 +49,7 @@
     <t/>
   </si>
   <si>
-    <t>["carousel-hero","columns-featured","columns-featured","cards-teaser","cards-teaser","hero-promo","hero-promo"]</t>
+    <t>["carousel-hero","columns-featured","columns-featured","article-list","article-list","hero-promo","hero-promo"]</t>
   </si>
   <si>
     <t>us/en</t>
@@ -61,7 +61,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-08-06T08:09:21.761Z</t>
+    <t>2026-08-06T19:05:35.144Z</t>
   </si>
   <si>
     <t>WKND Adventures and Travel</t>
@@ -82,7 +82,7 @@
     <t>about-us</t>
   </si>
   <si>
-    <t>2026-08-06T08:10:03.070Z</t>
+    <t>2026-08-06T19:17:25.706Z</t>
   </si>
   <si>
     <t>About Us</t>
@@ -94,7 +94,7 @@
     <t>us/en/adventures.report.json</t>
   </si>
   <si>
-    <t>["hero-intro","hero-intro","cards-teaser","cards-teaser","cards-teaser","cards-teaser","cards-teaser","cards-teaser","cards-teaser"]</t>
+    <t>["hero-promo","hero-promo","article-list"]</t>
   </si>
   <si>
     <t>us/en/adventures</t>
@@ -103,7 +103,7 @@
     <t>adventure-listing</t>
   </si>
   <si>
-    <t>2026-08-06T08:10:07.880Z</t>
+    <t>2026-08-07T03:09:28.549Z</t>
   </si>
   <si>
     <t>Adventures</t>
@@ -145,7 +145,7 @@
     <t>magazine-landing</t>
   </si>
   <si>
-    <t>2026-08-06T08:09:58.122Z</t>
+    <t>2026-08-07T06:49:39.094Z</t>
   </si>
   <si>
     <t>Magazine</t>
@@ -166,7 +166,7 @@
     <t>adventure-detail</t>
   </si>
   <si>
-    <t>2026-08-06T08:10:47.301Z</t>
+    <t>2026-08-07T03:52:36.551Z</t>
   </si>
   <si>
     <t>Bali Surf Camp</t>
@@ -181,7 +181,7 @@
     <t>us/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-08-06T08:10:53.657Z</t>
+    <t>2026-08-07T03:52:41.602Z</t>
   </si>
   <si>
     <t>Beervana in Portland</t>
@@ -196,7 +196,7 @@
     <t>us/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-08-06T08:10:59.799Z</t>
+    <t>2026-08-07T03:52:47.314Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -211,7 +211,7 @@
     <t>us/en/adventures/colorado-rock-climbing</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:05.230Z</t>
+    <t>2026-08-07T03:52:51.830Z</t>
   </si>
   <si>
     <t>Colorado Rock Climbing</t>
@@ -226,7 +226,7 @@
     <t>us/en/adventures/cycling-southern-utah</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:10.049Z</t>
+    <t>2026-08-07T03:52:56.771Z</t>
   </si>
   <si>
     <t>Cycling Southern Utah</t>
@@ -241,7 +241,7 @@
     <t>us/en/adventures/cycling-tuscany</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:14.793Z</t>
+    <t>2026-08-07T03:53:02.103Z</t>
   </si>
   <si>
     <t>Cycling Tuscany</t>
@@ -256,7 +256,7 @@
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:21.514Z</t>
+    <t>2026-08-07T03:53:06.972Z</t>
   </si>
   <si>
     <t>Downhill Skiing Wyoming</t>
@@ -271,7 +271,7 @@
     <t>us/en/adventures/gastronomic-marais-tour</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:27.625Z</t>
+    <t>2026-08-07T03:53:11.981Z</t>
   </si>
   <si>
     <t>Gastronomic Marais Tour</t>
@@ -286,7 +286,7 @@
     <t>us/en/adventures/napa-wine-tasting</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:33.534Z</t>
+    <t>2026-08-07T03:53:16.988Z</t>
   </si>
   <si>
     <t>Napa Wine Tasting</t>
@@ -301,7 +301,7 @@
     <t>us/en/adventures/riverside-camping-australia</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:38.037Z</t>
+    <t>2026-08-07T03:53:21.395Z</t>
   </si>
   <si>
     <t>Riverside Camping</t>
@@ -316,7 +316,7 @@
     <t>us/en/adventures/ski-touring-mont-blanc</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:42.932Z</t>
+    <t>2026-08-07T03:53:25.566Z</t>
   </si>
   <si>
     <t>Ski Touring Mont Blanc</t>
@@ -331,7 +331,7 @@
     <t>us/en/adventures/surf-camp-costa-rica</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:48.059Z</t>
+    <t>2026-08-07T03:53:31.681Z</t>
   </si>
   <si>
     <t>Surf Camp in Costa Rica</t>
@@ -346,7 +346,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:52.326Z</t>
+    <t>2026-08-07T03:53:36.966Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -361,7 +361,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:57.335Z</t>
+    <t>2026-08-07T03:53:40.930Z</t>
   </si>
   <si>
     <t>West Coast Cycling</t>
@@ -376,7 +376,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-08-06T08:12:03.133Z</t>
+    <t>2026-08-07T03:53:46.408Z</t>
   </si>
   <si>
     <t>Whistler Mountain Biking</t>
@@ -391,7 +391,7 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-08-06T08:12:08.188Z</t>
+    <t>2026-08-07T03:53:52.237Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>
@@ -406,7 +406,7 @@
     <t>Jacob Wester</t>
   </si>
   <si>
-    <t>["article-author","cards-related"]</t>
+    <t>["article-author","article-list"]</t>
   </si>
   <si>
     <t>us/en/magazine/arctic-surfing</t>
@@ -418,7 +418,7 @@
     <t>magazine-article</t>
   </si>
   <si>
-    <t>2026-08-06T08:25:31.199Z</t>
+    <t>2026-08-07T09:21:57.335Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -439,7 +439,7 @@
     <t>2020-09-30</t>
   </si>
   <si>
-    <t>2026-08-06T08:25:35.320Z</t>
+    <t>2026-08-07T09:22:03.334Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -457,7 +457,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-08-06T08:25:39.721Z</t>
+    <t>2026-08-07T09:22:06.914Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -475,7 +475,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-08-06T08:25:43.664Z</t>
+    <t>2026-08-07T09:22:11.736Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -490,7 +490,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-08-06T08:25:49.650Z</t>
+    <t>2026-08-07T09:22:15.764Z</t>
   </si>
   <si>
     <t>Western Australia</t>

</xml_diff>

<commit_message>
chore(magazine): rebuild article bundle; re-import 5 articles with dynamic related
Related section now the self-excluding dynamic article-list (was stale
cards-related on published content). Content re-uploaded to DA.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-magazine-article.report.xlsx
+++ b/tools/importer/reports/import-magazine-article.report.xlsx
@@ -136,7 +136,7 @@
     <t>us/en/magazine.report.json</t>
   </si>
   <si>
-    <t>["columns-featured","columns-featured","article-list","cards-teaser","cards-teaser"]</t>
+    <t>["columns-featured","columns-featured","article-list","article-list-members","article-list-members"]</t>
   </si>
   <si>
     <t>us/en/magazine</t>
@@ -145,7 +145,7 @@
     <t>magazine-landing</t>
   </si>
   <si>
-    <t>2026-08-07T06:49:39.094Z</t>
+    <t>2026-08-07T10:26:33.120Z</t>
   </si>
   <si>
     <t>Magazine</t>
@@ -418,7 +418,7 @@
     <t>magazine-article</t>
   </si>
   <si>
-    <t>2026-08-07T09:21:57.335Z</t>
+    <t>2026-08-07T10:43:34.373Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -439,7 +439,7 @@
     <t>2020-09-30</t>
   </si>
   <si>
-    <t>2026-08-07T09:22:03.334Z</t>
+    <t>2026-08-07T10:43:38.619Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -457,7 +457,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-08-07T09:22:06.914Z</t>
+    <t>2026-08-07T10:43:43.607Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -475,7 +475,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-08-07T09:22:11.736Z</t>
+    <t>2026-08-07T10:43:48.819Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -490,7 +490,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-08-07T09:22:15.764Z</t>
+    <t>2026-08-07T10:43:54.002Z</t>
   </si>
   <si>
     <t>Western Australia</t>

</xml_diff>

<commit_message>
fix(magazine-article): breadcrumb, grey pull-quote, related sidebar list, author social icons
Critique fixes vs source:
- breadcrumb autoblock now also covers /magazine/{slug} (Magazine > Title), below lead image
- pull-quote renders in a grey #ebebeb box (Asar 36/54)
- related 'SHARE THIS STORY' now a title+date list with left accent + yellow hover (article-list related mode)
- author social links render as dark icon boxes (fb/twitter/insta), adopted from trailing siblings

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-magazine-article.report.xlsx
+++ b/tools/importer/reports/import-magazine-article.report.xlsx
@@ -418,7 +418,7 @@
     <t>magazine-article</t>
   </si>
   <si>
-    <t>2026-08-07T10:43:34.373Z</t>
+    <t>2026-08-07T12:18:42.590Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -439,7 +439,7 @@
     <t>2020-09-30</t>
   </si>
   <si>
-    <t>2026-08-07T10:43:38.619Z</t>
+    <t>2026-08-07T12:18:48.179Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -457,7 +457,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-08-07T10:43:43.607Z</t>
+    <t>2026-08-07T12:18:53.759Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -475,7 +475,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-08-07T10:43:48.819Z</t>
+    <t>2026-08-07T12:18:58.899Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -490,7 +490,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-08-07T10:43:54.002Z</t>
+    <t>2026-08-07T12:19:04.623Z</t>
   </si>
   <si>
     <t>Western Australia</t>

</xml_diff>